<commit_message>
docs: propagate per-partner rounding to WBS, backlog (+12 tickets), service map, addendum
- WBS WPs 3.2/3.3/4.8/5.5/7.3/10.3/15.3 annotated
- 12 new tickets across config-registry/txn/payment-executor/revenue-ledger/admin-ui/qa
- ADDENDUM-001 (spec deltas) + MASTER_PLAN change log

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/GMEPay+_WBS.xlsx
+++ b/Documentation/GMEPay+_WBS.xlsx
@@ -1421,7 +1421,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Entity model</t>
+          <t>Entity model; + Partner.settlement_rounding_mode field</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Txn schema</t>
+          <t>Txn schema; + locked booked_settlement_amount &amp; rounding_mode &amp; residual</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Commit logic</t>
+          <t>Commit logic; + book settlement under partner rule, lock on txn, post residual</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>Revenue capture</t>
+          <t>Revenue capture; + rounding-residual posting to REVENUE_ROUNDING</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="K71" s="8" t="inlineStr">
         <is>
-          <t>Partner UI</t>
+          <t>Partner UI; + settlement-rounding-mode setting on partner</t>
         </is>
       </c>
       <c r="L71" s="8" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="K112" s="4" t="inlineStr">
         <is>
-          <t>Vector results</t>
+          <t>Vector results; + rounding-residual reconciliation tests</t>
         </is>
       </c>
       <c r="L112" s="4" t="inlineStr">

</xml_diff>